<commit_message>
corrige robo e atualizar planilha
</commit_message>
<xml_diff>
--- a/app_zenite/PRECIFICAÇÃO IPHONE.xlsx
+++ b/app_zenite/PRECIFICAÇÃO IPHONE.xlsx
@@ -182,10 +182,10 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -967,8 +967,8 @@
     <col width="29" customWidth="1" style="3" min="7" max="7"/>
     <col width="17.88671875" customWidth="1" style="3" min="8" max="8"/>
     <col width="25.77734375" bestFit="1" customWidth="1" style="3" min="9" max="9"/>
-    <col width="8.88671875" customWidth="1" style="3" min="10" max="15"/>
-    <col width="8.88671875" customWidth="1" style="3" min="16" max="16384"/>
+    <col width="8.88671875" customWidth="1" style="3" min="10" max="16"/>
+    <col width="8.88671875" customWidth="1" style="3" min="17" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="21" customHeight="1">
@@ -1030,7 +1030,7 @@
         </is>
       </c>
       <c r="C2" s="13" t="n">
-        <v>3550</v>
+        <v>3450</v>
       </c>
       <c r="D2" s="13" t="n">
         <v>150</v>
@@ -1065,7 +1065,7 @@
         </is>
       </c>
       <c r="C3" s="13" t="n">
-        <v>3900</v>
+        <v>3899</v>
       </c>
       <c r="D3" s="13" t="n">
         <v>150</v>
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="C4" s="13" t="n">
-        <v>4500</v>
+        <v>0</v>
       </c>
       <c r="D4" s="13" t="n">
         <v>150</v>
@@ -1170,7 +1170,7 @@
         </is>
       </c>
       <c r="C6" s="13" t="n">
-        <v>3799</v>
+        <v>3299</v>
       </c>
       <c r="D6" s="13" t="n">
         <v>150</v>
@@ -1240,7 +1240,7 @@
         </is>
       </c>
       <c r="C8" s="13" t="n">
-        <v>5300</v>
+        <v>5350</v>
       </c>
       <c r="D8" s="13" t="n">
         <v>150</v>
@@ -1275,7 +1275,7 @@
         </is>
       </c>
       <c r="C9" s="13" t="n">
-        <v>0</v>
+        <v>6699</v>
       </c>
       <c r="D9" s="13" t="n">
         <v>150</v>
@@ -1310,7 +1310,7 @@
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>0</v>
+        <v>6699</v>
       </c>
       <c r="D10" s="13" t="n">
         <v>150</v>
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="C11" s="13" t="n">
-        <v>7450</v>
+        <v>7050</v>
       </c>
       <c r="D11" s="13" t="n">
         <v>150</v>
@@ -1380,7 +1380,7 @@
         </is>
       </c>
       <c r="C12" s="13" t="n">
-        <v>3550</v>
+        <v>3400</v>
       </c>
       <c r="D12" s="13" t="n">
         <v>150</v>
@@ -1415,7 +1415,7 @@
         </is>
       </c>
       <c r="C13" s="13" t="n">
-        <v>4200</v>
+        <v>4150</v>
       </c>
       <c r="D13" s="13" t="n">
         <v>150</v>
@@ -1450,7 +1450,7 @@
         </is>
       </c>
       <c r="C14" s="13" t="n">
-        <v>6950</v>
+        <v>6650</v>
       </c>
       <c r="D14" s="13" t="n">
         <v>150</v>
@@ -1520,7 +1520,7 @@
         </is>
       </c>
       <c r="C16" s="13" t="n">
-        <v>8800</v>
+        <v>8100</v>
       </c>
       <c r="D16" s="13" t="n">
         <v>150</v>
@@ -1555,7 +1555,7 @@
         </is>
       </c>
       <c r="C17" s="13" t="n">
-        <v>7500</v>
+        <v>6950</v>
       </c>
       <c r="D17" s="13" t="n">
         <v>150</v>
@@ -1590,7 +1590,7 @@
         </is>
       </c>
       <c r="C18" s="13" t="n">
-        <v>8500</v>
+        <v>8480</v>
       </c>
       <c r="D18" s="13" t="n">
         <v>150</v>
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="C19" s="13" t="n">
-        <v>9400</v>
+        <v>9340</v>
       </c>
       <c r="D19" s="13" t="n">
         <v>150</v>
@@ -1660,7 +1660,7 @@
         </is>
       </c>
       <c r="C20" s="13" t="n">
-        <v>11200</v>
+        <v>11150</v>
       </c>
       <c r="D20" s="13" t="n">
         <v>150</v>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="B21" s="1" t="inlineStr"/>
       <c r="C21" s="13" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="D21" s="13" t="n">
         <v>150</v>
@@ -1718,7 +1718,7 @@
       </c>
       <c r="B22" s="1" t="inlineStr"/>
       <c r="C22" s="13" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="D22" s="13" t="n">
         <v>150</v>
@@ -1747,7 +1747,7 @@
       </c>
       <c r="B23" s="1" t="inlineStr"/>
       <c r="C23" s="13" t="n">
-        <v>1700</v>
+        <v>0</v>
       </c>
       <c r="D23" s="13" t="n">
         <v>150</v>
@@ -1892,7 +1892,7 @@
       </c>
       <c r="B28" s="1" t="inlineStr"/>
       <c r="C28" s="13" t="n">
-        <v>4750</v>
+        <v>4850</v>
       </c>
       <c r="D28" s="13" t="n">
         <v>150</v>
@@ -1950,7 +1950,7 @@
       </c>
       <c r="B30" s="1" t="inlineStr"/>
       <c r="C30" s="13" t="n">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="D30" s="13" t="n">
         <v>150</v>
@@ -1979,7 +1979,7 @@
       </c>
       <c r="B31" s="1" t="inlineStr"/>
       <c r="C31" s="13" t="n">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="D31" s="13" t="n">
         <v>150</v>
@@ -2037,7 +2037,7 @@
       </c>
       <c r="B33" s="1" t="inlineStr"/>
       <c r="C33" s="13" t="n">
-        <v>1350</v>
+        <v>1299</v>
       </c>
       <c r="D33" s="13" t="n">
         <v>150</v>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="B34" s="1" t="inlineStr"/>
       <c r="C34" s="13" t="n">
-        <v>1350</v>
+        <v>1300</v>
       </c>
       <c r="D34" s="13" t="n">
         <v>150</v>
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="C35" s="13" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="D35" s="13" t="n">
         <v>150</v>
@@ -2165,7 +2165,7 @@
         </is>
       </c>
       <c r="C37" s="13" t="n">
-        <v>3850</v>
+        <v>3900</v>
       </c>
       <c r="D37" s="13" t="n">
         <v>150</v>
@@ -2198,7 +2198,7 @@
         </is>
       </c>
       <c r="C38" s="13" t="n">
-        <v>4650</v>
+        <v>4600</v>
       </c>
       <c r="D38" s="13" t="n">
         <v>150</v>
@@ -2231,7 +2231,7 @@
         </is>
       </c>
       <c r="C39" s="13" t="n">
-        <v>5850</v>
+        <v>5849</v>
       </c>
       <c r="D39" s="13" t="n">
         <v>150</v>
@@ -2264,7 +2264,7 @@
         </is>
       </c>
       <c r="C40" s="13" t="n">
-        <v>6150</v>
+        <v>6400</v>
       </c>
       <c r="D40" s="13" t="n">
         <v>150</v>
@@ -2297,7 +2297,7 @@
         </is>
       </c>
       <c r="C41" s="13" t="n">
-        <v>7200</v>
+        <v>0</v>
       </c>
       <c r="D41" s="13" t="n">
         <v>150</v>
@@ -2363,7 +2363,7 @@
         </is>
       </c>
       <c r="C43" s="13" t="n">
-        <v>6300</v>
+        <v>6250</v>
       </c>
       <c r="D43" s="13" t="n">
         <v>150</v>
@@ -2396,7 +2396,7 @@
         </is>
       </c>
       <c r="C44" s="13" t="n">
-        <v>10700</v>
+        <v>7550</v>
       </c>
       <c r="D44" s="13" t="n">
         <v>150</v>
@@ -2462,7 +2462,7 @@
         </is>
       </c>
       <c r="C46" s="13" t="n">
-        <v>6500</v>
+        <v>0</v>
       </c>
       <c r="D46" s="13" t="n">
         <v>150</v>
@@ -2561,7 +2561,7 @@
         </is>
       </c>
       <c r="C49" s="13" t="n">
-        <v>10200</v>
+        <v>13299</v>
       </c>
       <c r="D49" s="13" t="n">
         <v>150</v>
@@ -2594,7 +2594,7 @@
         </is>
       </c>
       <c r="C50" s="13" t="n">
-        <v>0</v>
+        <v>14800</v>
       </c>
       <c r="D50" s="13" t="n">
         <v>150</v>

</xml_diff>